<commit_message>
Remove temporary Excel file and update plots notebook with new queries and improved data handling. Added field categorization for evaluation results in the RAG evaluator and modified JSON output format.
</commit_message>
<xml_diff>
--- a/RAG eval.xlsx
+++ b/RAG eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\EnergeticGraph\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363E6514-ABE2-4E3F-9577-D7C873D2512D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA32935A-C876-4BF6-9E09-4BC8AD580BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31635" yWindow="13500" windowWidth="43200" windowHeight="23445" xr2:uid="{BC529AF5-19B5-479C-B76B-AB0B51AFE937}"/>
+    <workbookView xWindow="4515" yWindow="12495" windowWidth="43200" windowHeight="23445" xr2:uid="{BC529AF5-19B5-479C-B76B-AB0B51AFE937}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>precision@1</t>
   </si>
@@ -80,7 +80,13 @@
     <t>jonghyunlee/ChemBERT_ChEMBL_pretrained</t>
   </si>
   <si>
-    <t>* cosine similarity &gt; 0.95</t>
+    <t>* cosine similarity &gt;= 0.95</t>
+  </si>
+  <si>
+    <t>10 queries</t>
+  </si>
+  <si>
+    <t>50 queries</t>
   </si>
 </sst>
 </file>
@@ -143,6 +149,1079 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-IL"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>10 queries</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:strRef>
+              <c:f>Sheet1!$A$3:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>precision@1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>precision@2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>precision@3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>precision@4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>precision@5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>precision@6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>precision@7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>precision@8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>precision@9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>precision@10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$3:$B$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0.88900000000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.77800000000000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.70399999999999996</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.61099999999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.55600000000000005</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.51900000000000002</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.49199999999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.47199999999999998</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.45700000000000002</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.44400000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5C20-45CF-81EC-349CB9577ED6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$D$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>50 queries</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:strRef>
+              <c:f>Sheet1!$A$3:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>precision@1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>precision@2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>precision@3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>precision@4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>precision@5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>precision@6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>precision@7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>precision@8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>precision@9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>precision@10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$D$3:$D$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0.90700000000000003</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.87</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.84599999999999997</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.82399999999999995</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.80700000000000005</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.79300000000000004</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.78</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.76600000000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.755</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.74399999999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5C20-45CF-81EC-349CB9577ED6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="95759200"/>
+        <c:axId val="95759680"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="95759200"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="95759680"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="95759680"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="95759200"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-IL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>552449</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>157161</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8EF7165E-26FF-3399-EE6C-FCD7350C38FB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -462,16 +1541,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12A3ED85-D83C-41B6-9201-C96BA5660DCF}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="3.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -482,6 +1556,10 @@
         <v>13</v>
       </c>
       <c r="C1" s="2"/>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -513,6 +1591,12 @@
       <c r="C3">
         <v>0.314</v>
       </c>
+      <c r="D3">
+        <v>0.90700000000000003</v>
+      </c>
+      <c r="E3">
+        <v>0.28999999999999998</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -524,6 +1608,12 @@
       <c r="C4">
         <v>0.34200000000000003</v>
       </c>
+      <c r="D4">
+        <v>0.87</v>
+      </c>
+      <c r="E4">
+        <v>0.307</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -535,6 +1625,12 @@
       <c r="C5">
         <v>0.36699999999999999</v>
       </c>
+      <c r="D5">
+        <v>0.84599999999999997</v>
+      </c>
+      <c r="E5">
+        <v>0.32500000000000001</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -546,6 +1642,12 @@
       <c r="C6">
         <v>0.65600000000000003</v>
       </c>
+      <c r="D6">
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="E6">
+        <v>0.32900000000000001</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -557,6 +1659,12 @@
       <c r="C7">
         <v>0.36199999999999999</v>
       </c>
+      <c r="D7">
+        <v>0.80700000000000005</v>
+      </c>
+      <c r="E7">
+        <v>0.34200000000000003</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -568,6 +1676,12 @@
       <c r="C8">
         <v>0.372</v>
       </c>
+      <c r="D8">
+        <v>0.79300000000000004</v>
+      </c>
+      <c r="E8">
+        <v>0.35399999999999998</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -579,6 +1693,12 @@
       <c r="C9">
         <v>0.38200000000000001</v>
       </c>
+      <c r="D9">
+        <v>0.78</v>
+      </c>
+      <c r="E9">
+        <v>0.36299999999999999</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -590,6 +1710,12 @@
       <c r="C10">
         <v>0.39</v>
       </c>
+      <c r="D10">
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="E10">
+        <v>0.37</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -601,6 +1727,12 @@
       <c r="C11">
         <v>0.39700000000000002</v>
       </c>
+      <c r="D11">
+        <v>0.755</v>
+      </c>
+      <c r="E11">
+        <v>0.376</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -612,18 +1744,38 @@
       <c r="C12">
         <v>0.40300000000000002</v>
       </c>
+      <c r="D12">
+        <v>0.74399999999999999</v>
+      </c>
+      <c r="E12">
+        <v>0.38</v>
+      </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>